<commit_message>
Add scene sheet loop controls
</commit_message>
<xml_diff>
--- a/Feuilles/A bout.xlsx
+++ b/Feuilles/A bout.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanaismusic/Documents/CLIC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanaismusic/Documents/CLIC/Feuilles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A1D9FF-D96D-B043-B0EA-88762AC2C3FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB4DC93A-6C3A-EC4A-BAA5-994B1DED618A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10360" yWindow="2140" windowWidth="28040" windowHeight="17440" xr2:uid="{2F1647A4-8C84-E14B-83BA-CB692A19D8A6}"/>
+    <workbookView xWindow="6080" yWindow="2140" windowWidth="28040" windowHeight="17440" xr2:uid="{2F1647A4-8C84-E14B-83BA-CB692A19D8A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>MES</t>
   </si>
@@ -77,9 +77,6 @@
     <t>COUPLET 3</t>
   </si>
   <si>
-    <t>Ha Ha Ha…</t>
-  </si>
-  <si>
     <t>PONT FX</t>
   </si>
   <si>
@@ -89,14 +86,20 @@
     <t>AD LIB</t>
   </si>
   <si>
-    <t>Ha Ha Ha Ha…</t>
+    <t>LOOP</t>
+  </si>
+  <si>
+    <t>Ha Ha Ha... B</t>
+  </si>
+  <si>
+    <t>Ha Ha Ha... A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -109,6 +112,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -132,9 +142,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -469,10 +480,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85B34C31-2D9C-7940-9F39-E67ACD52E89F}">
-  <dimension ref="A1:D224"/>
+  <dimension ref="A1:E224"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="11.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -485,8 +499,11 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -500,7 +517,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -511,7 +528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -522,7 +539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -533,7 +550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -544,7 +561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -555,7 +572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -566,7 +583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -577,7 +594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -588,7 +605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -599,7 +616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -610,7 +627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -621,7 +638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -632,7 +649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -643,7 +660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -788,8 +805,8 @@
       <c r="C28">
         <v>0</v>
       </c>
-      <c r="D28" t="s">
-        <v>12</v>
+      <c r="D28" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -1117,7 +1134,7 @@
         <v>0</v>
       </c>
       <c r="D57" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
@@ -1208,7 +1225,7 @@
         <v>1</v>
       </c>
       <c r="D65" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
@@ -1586,7 +1603,7 @@
         <v>0</v>
       </c>
       <c r="D98" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>